<commit_message>
Adiciona relatorio final gerado em Excel
</commit_message>
<xml_diff>
--- a/Relatorio_Final_Analisado.xlsx
+++ b/Relatorio_Final_Analisado.xlsx
@@ -725,6 +725,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="A1" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Opção 1, Opção 2"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove linha com aviso de tipagem do Pylance
</commit_message>
<xml_diff>
--- a/Relatorio_Final_Analisado.xlsx
+++ b/Relatorio_Final_Analisado.xlsx
@@ -679,7 +679,7 @@
         <v>101</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>3905</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -692,7 +692,7 @@
         <v>50</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>8420</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -705,7 +705,7 @@
         <v>68</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>5585</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -718,18 +718,13 @@
         <v>219</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>17910</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="A1" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Opção 1, Opção 2"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>